<commit_message>
Idk its been a while... log model plots
</commit_message>
<xml_diff>
--- a/Single sheet May2023 Data.xlsx
+++ b/Single sheet May2023 Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heref\Documents\UW Madison Files\Project Stuff\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heref\Documents\Project stuff\LucasProject\Repo_Backup\Project_code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17604571-65B4-4927-988B-9F613E259A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00CA4BE-EAC7-482E-8543-B5963448F61D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{B2BB9978-D008-4886-AD29-AD3E6970A3E0}"/>
+    <workbookView xWindow="-12105" yWindow="-3900" windowWidth="12210" windowHeight="12885" activeTab="1" xr2:uid="{B2BB9978-D008-4886-AD29-AD3E6970A3E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -298,14 +298,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -643,177 +642,165 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E27A5A1E-CE4A-441F-B2B9-A3107CDC5860}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5">
         <v>39</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5">
         <v>0.23877614949795342</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5">
         <v>6.1224653717423952E-3</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5">
         <v>5.4937261264824307E-6</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6">
         <v>71</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6">
         <v>0.54928979571594061</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6">
         <v>7.7364759959991638E-3</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6">
         <v>2.6705201981185646E-6</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="4">
         <v>16</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <v>6.4935064363996473E-2</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>4.0584415227497795E-3</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <v>1.3250689753439367E-6</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12">
         <v>2.0031291525330795E-4</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12">
         <v>2</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12">
         <v>1.0015645762665397E-4</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12">
         <v>29.643921572674078</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12">
         <v>3.1086040889228957E-11</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12">
         <v>3.0698942378503262</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>63</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13">
         <v>4.155740413047909E-4</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13">
         <v>123</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13">
         <v>3.378650742315373E-6</v>
       </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-    </row>
-    <row r="15" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+    </row>
+    <row r="15" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="4">
         <v>6.1588695655809885E-4</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="4">
         <v>125</v>
       </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -824,9 +811,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11F99FF0-2235-4DA3-8ED8-44AD23702AC2}">
   <dimension ref="B1:X127"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -888,7 +875,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>6</v>
       </c>
@@ -950,7 +937,7 @@
         <v>2.1540893888719959E-3</v>
       </c>
     </row>
-    <row r="3" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>7</v>
       </c>
@@ -1015,7 +1002,7 @@
         <v>2.6541458541458523E-3</v>
       </c>
     </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -1081,7 +1068,7 @@
         <v>2.7411670296916164E-3</v>
       </c>
     </row>
-    <row r="5" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>7</v>
       </c>
@@ -1143,7 +1130,7 @@
         <v>4.6043660687138926E-3</v>
       </c>
     </row>
-    <row r="6" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>6</v>
       </c>
@@ -1208,7 +1195,7 @@
         <v>3.7158041958041945E-3</v>
       </c>
     </row>
-    <row r="7" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>7</v>
       </c>
@@ -1274,7 +1261,7 @@
         <v>5.5737062937063148E-3</v>
       </c>
     </row>
-    <row r="8" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>6</v>
       </c>
@@ -1336,7 +1323,7 @@
         <v>4.9262555626191995E-3</v>
       </c>
     </row>
-    <row r="9" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>7</v>
       </c>
@@ -1401,7 +1388,7 @@
         <v>4.2723281250000023E-3</v>
       </c>
     </row>
-    <row r="10" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>6</v>
       </c>
@@ -1467,7 +1454,7 @@
         <v>3.3942770831585146E-3</v>
       </c>
     </row>
-    <row r="11" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>7</v>
       </c>
@@ -1529,7 +1516,7 @@
         <v>4.7151933962264192E-3</v>
       </c>
     </row>
-    <row r="12" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>6</v>
       </c>
@@ -1591,7 +1578,7 @@
         <v>3.2661911554921512E-3</v>
       </c>
     </row>
-    <row r="13" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>7</v>
       </c>
@@ -1653,7 +1640,7 @@
         <v>4.7420048076923021E-3</v>
       </c>
     </row>
-    <row r="14" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>7</v>
       </c>
@@ -1715,7 +1702,7 @@
         <v>4.0199275759903435E-3</v>
       </c>
     </row>
-    <row r="15" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>6</v>
       </c>
@@ -1777,7 +1764,7 @@
         <v>3.6487180475768162E-3</v>
       </c>
     </row>
-    <row r="16" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>6</v>
       </c>
@@ -1839,7 +1826,7 @@
         <v>6.6745588235293928E-3</v>
       </c>
     </row>
-    <row r="17" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>7</v>
       </c>
@@ -1901,7 +1888,7 @@
         <v>3.8323309557774621E-3</v>
       </c>
     </row>
-    <row r="18" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>8</v>
       </c>
@@ -1960,7 +1947,7 @@
         <v>8.3226457590876782E-3</v>
       </c>
     </row>
-    <row r="19" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>9</v>
       </c>
@@ -2019,7 +2006,7 @@
         <v>3.9149065743944575E-3</v>
       </c>
     </row>
-    <row r="20" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>10</v>
       </c>
@@ -2078,7 +2065,7 @@
         <v>9.045566433566422E-3</v>
       </c>
     </row>
-    <row r="21" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>8</v>
       </c>
@@ -2137,7 +2124,7 @@
         <v>6.0018550724637611E-3</v>
       </c>
     </row>
-    <row r="22" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>9</v>
       </c>
@@ -2196,7 +2183,7 @@
         <v>6.2079999999999922E-3</v>
       </c>
     </row>
-    <row r="23" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>10</v>
       </c>
@@ -2255,7 +2242,7 @@
         <v>7.037333333333326E-3</v>
       </c>
     </row>
-    <row r="24" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>8</v>
       </c>
@@ -2314,7 +2301,7 @@
         <v>6.7993043478261021E-3</v>
       </c>
     </row>
-    <row r="25" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>9</v>
       </c>
@@ -2373,7 +2360,7 @@
         <v>6.9125524296675478E-3</v>
       </c>
     </row>
-    <row r="26" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>10</v>
       </c>
@@ -2432,7 +2419,7 @@
         <v>6.1630328820116058E-3</v>
       </c>
     </row>
-    <row r="27" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>8</v>
       </c>
@@ -2491,7 +2478,7 @@
         <v>6.9503999999999989E-3</v>
       </c>
     </row>
-    <row r="28" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>9</v>
       </c>
@@ -2550,7 +2537,7 @@
         <v>1.192713472485772E-2</v>
       </c>
     </row>
-    <row r="29" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
         <v>10</v>
       </c>
@@ -2609,7 +2596,7 @@
         <v>9.258228739002965E-3</v>
       </c>
     </row>
-    <row r="30" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>8</v>
       </c>
@@ -2668,7 +2655,7 @@
         <v>6.8748521739130687E-3</v>
       </c>
     </row>
-    <row r="31" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>9</v>
       </c>
@@ -2727,7 +2714,7 @@
         <v>6.8967619047619272E-3</v>
       </c>
     </row>
-    <row r="32" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>10</v>
       </c>
@@ -2786,7 +2773,7 @@
         <v>9.8308571428571429E-3</v>
       </c>
     </row>
-    <row r="33" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>8</v>
       </c>
@@ -2845,7 +2832,7 @@
         <v>6.9470151975684147E-3</v>
       </c>
     </row>
-    <row r="34" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>9</v>
       </c>
@@ -2904,7 +2891,7 @@
         <v>9.9615584415584379E-3</v>
       </c>
     </row>
-    <row r="35" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>10</v>
       </c>
@@ -2963,7 +2950,7 @@
         <v>7.2217600000000033E-3</v>
       </c>
     </row>
-    <row r="36" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>11</v>
       </c>
@@ -3022,7 +3009,7 @@
         <v>8.1333551020408203E-3</v>
       </c>
     </row>
-    <row r="37" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>11</v>
       </c>
@@ -3081,7 +3068,7 @@
         <v>6.8943523404255136E-3</v>
       </c>
     </row>
-    <row r="38" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>11</v>
       </c>
@@ -3140,7 +3127,7 @@
         <v>8.3184872727273037E-3</v>
       </c>
     </row>
-    <row r="39" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>11</v>
       </c>
@@ -3199,7 +3186,7 @@
         <v>6.7314285714285783E-3</v>
       </c>
     </row>
-    <row r="40" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>11</v>
       </c>
@@ -3258,7 +3245,7 @@
         <v>8.1600000000000058E-3</v>
       </c>
     </row>
-    <row r="41" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>12</v>
       </c>
@@ -3314,7 +3301,7 @@
         <v>7.7284578136463675E-3</v>
       </c>
     </row>
-    <row r="42" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>13</v>
       </c>
@@ -3370,7 +3357,7 @@
         <v>1.0947611285266459E-2</v>
       </c>
     </row>
-    <row r="43" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>14</v>
       </c>
@@ -3426,7 +3413,7 @@
         <v>6.4074830769230758E-3</v>
       </c>
     </row>
-    <row r="44" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>14</v>
       </c>
@@ -3482,7 +3469,7 @@
         <v>5.7845106382978725E-3</v>
       </c>
     </row>
-    <row r="45" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>12</v>
       </c>
@@ -3538,7 +3525,7 @@
         <v>9.3658181818181765E-3</v>
       </c>
     </row>
-    <row r="46" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>13</v>
       </c>
@@ -3594,7 +3581,7 @@
         <v>5.2039344262295112E-3</v>
       </c>
     </row>
-    <row r="47" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>12</v>
       </c>
@@ -3650,7 +3637,7 @@
         <v>5.8575238095238159E-3</v>
       </c>
     </row>
-    <row r="48" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>14</v>
       </c>
@@ -3706,7 +3693,7 @@
         <v>5.2697806451612889E-3</v>
       </c>
     </row>
-    <row r="49" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>14</v>
       </c>
@@ -3762,7 +3749,7 @@
         <v>7.3164255319149015E-3</v>
       </c>
     </row>
-    <row r="50" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
         <v>12</v>
       </c>
@@ -3818,7 +3805,7 @@
         <v>5.2629482517482524E-3</v>
       </c>
     </row>
-    <row r="51" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
         <v>13</v>
       </c>
@@ -3874,7 +3861,7 @@
         <v>6.3299047619047579E-3</v>
       </c>
     </row>
-    <row r="52" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>12</v>
       </c>
@@ -3930,7 +3917,7 @@
         <v>9.4034285714285661E-3</v>
       </c>
     </row>
-    <row r="53" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
         <v>14</v>
       </c>
@@ -3986,7 +3973,7 @@
         <v>8.3378797409805749E-3</v>
       </c>
     </row>
-    <row r="54" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
         <v>13</v>
       </c>
@@ -4042,7 +4029,7 @@
         <v>6.5454545454545453E-3</v>
       </c>
     </row>
-    <row r="55" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>12</v>
       </c>
@@ -4098,7 +4085,7 @@
         <v>8.1504864864864815E-3</v>
       </c>
     </row>
-    <row r="56" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>13</v>
       </c>
@@ -4154,7 +4141,7 @@
         <v>1.0091935135135129E-2</v>
       </c>
     </row>
-    <row r="57" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>14</v>
       </c>
@@ -4210,7 +4197,7 @@
         <v>7.5544367301231723E-3</v>
       </c>
     </row>
-    <row r="58" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>12</v>
       </c>
@@ -4266,7 +4253,7 @@
         <v>9.520535885167462E-3</v>
       </c>
     </row>
-    <row r="59" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>13</v>
       </c>
@@ -4322,7 +4309,7 @@
         <v>8.6855111111111133E-3</v>
       </c>
     </row>
-    <row r="60" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
         <v>14</v>
       </c>
@@ -4378,7 +4365,7 @@
         <v>9.778110638297869E-3</v>
       </c>
     </row>
-    <row r="61" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B61" t="s">
         <v>12</v>
       </c>
@@ -4434,7 +4421,7 @@
         <v>8.4756786799826331E-3</v>
       </c>
     </row>
-    <row r="62" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
         <v>13</v>
       </c>
@@ -4490,7 +4477,7 @@
         <v>8.2873469387754872E-3</v>
       </c>
     </row>
-    <row r="63" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
         <v>14</v>
       </c>
@@ -4546,7 +4533,7 @@
         <v>6.9284833068362422E-3</v>
       </c>
     </row>
-    <row r="64" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
         <v>12</v>
       </c>
@@ -4602,7 +4589,7 @@
         <v>6.8520452830188663E-3</v>
       </c>
     </row>
-    <row r="65" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
         <v>13</v>
       </c>
@@ -4658,7 +4645,7 @@
         <v>7.820940336562986E-3</v>
       </c>
     </row>
-    <row r="66" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
         <v>14</v>
       </c>
@@ -4714,7 +4701,7 @@
         <v>7.8665890909090964E-3</v>
       </c>
     </row>
-    <row r="67" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>12</v>
       </c>
@@ -4770,7 +4757,7 @@
         <v>8.1375135135135206E-3</v>
       </c>
     </row>
-    <row r="68" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>13</v>
       </c>
@@ -4826,7 +4813,7 @@
         <v>7.5822545454545514E-3</v>
       </c>
     </row>
-    <row r="69" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>14</v>
       </c>
@@ -4882,7 +4869,7 @@
         <v>8.8815021337126671E-3</v>
       </c>
     </row>
-    <row r="70" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>15</v>
       </c>
@@ -4938,7 +4925,7 @@
         <v>7.7969230769230763E-3</v>
       </c>
     </row>
-    <row r="71" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
         <v>16</v>
       </c>
@@ -4994,7 +4981,7 @@
         <v>7.4424092664092684E-3</v>
       </c>
     </row>
-    <row r="72" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>17</v>
       </c>
@@ -5050,7 +5037,7 @@
         <v>7.8703058823529209E-3</v>
       </c>
     </row>
-    <row r="73" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B73" t="s">
         <v>18</v>
       </c>
@@ -5103,7 +5090,7 @@
         <v>19.350000000000001</v>
       </c>
     </row>
-    <row r="74" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B74" t="s">
         <v>15</v>
       </c>
@@ -5156,7 +5143,7 @@
         <v>18.55</v>
       </c>
     </row>
-    <row r="75" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B75" t="s">
         <v>16</v>
       </c>
@@ -5209,7 +5196,7 @@
         <v>18.649999999999999</v>
       </c>
     </row>
-    <row r="76" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B76" t="s">
         <v>17</v>
       </c>
@@ -5262,7 +5249,7 @@
         <v>18.799999999999997</v>
       </c>
     </row>
-    <row r="77" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
         <v>18</v>
       </c>
@@ -5315,7 +5302,7 @@
         <v>18.799999999999997</v>
       </c>
     </row>
-    <row r="78" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>15</v>
       </c>
@@ -5368,7 +5355,7 @@
         <v>14.75</v>
       </c>
     </row>
-    <row r="79" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
         <v>16</v>
       </c>
@@ -5421,7 +5408,7 @@
         <v>14.75</v>
       </c>
     </row>
-    <row r="80" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
         <v>17</v>
       </c>
@@ -5474,7 +5461,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="81" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
         <v>18</v>
       </c>
@@ -5527,7 +5514,7 @@
         <v>14.75</v>
       </c>
     </row>
-    <row r="82" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
         <v>16</v>
       </c>
@@ -5580,7 +5567,7 @@
         <v>14.6</v>
       </c>
     </row>
-    <row r="83" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
         <v>17</v>
       </c>
@@ -5633,7 +5620,7 @@
         <v>14.55</v>
       </c>
     </row>
-    <row r="84" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
         <v>18</v>
       </c>
@@ -5686,7 +5673,7 @@
         <v>14.65</v>
       </c>
     </row>
-    <row r="85" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>15</v>
       </c>
@@ -5739,7 +5726,7 @@
         <v>14.6</v>
       </c>
     </row>
-    <row r="86" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>15</v>
       </c>
@@ -5792,7 +5779,7 @@
         <v>15.55</v>
       </c>
     </row>
-    <row r="87" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>16</v>
       </c>
@@ -5845,7 +5832,7 @@
         <v>15.600000000000001</v>
       </c>
     </row>
-    <row r="88" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
         <v>17</v>
       </c>
@@ -5898,7 +5885,7 @@
         <v>15.6</v>
       </c>
     </row>
-    <row r="89" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B89" t="s">
         <v>18</v>
       </c>
@@ -5951,7 +5938,7 @@
         <v>15.6</v>
       </c>
     </row>
-    <row r="90" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>15</v>
       </c>
@@ -6004,7 +5991,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="91" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>16</v>
       </c>
@@ -6057,7 +6044,7 @@
         <v>16.950000000000003</v>
       </c>
     </row>
-    <row r="92" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B92" t="s">
         <v>17</v>
       </c>
@@ -6110,7 +6097,7 @@
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="93" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>18</v>
       </c>
@@ -6163,7 +6150,7 @@
         <v>17.05</v>
       </c>
     </row>
-    <row r="94" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>15</v>
       </c>
@@ -6216,7 +6203,7 @@
         <v>18.649999999999999</v>
       </c>
     </row>
-    <row r="95" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>16</v>
       </c>
@@ -6269,7 +6256,7 @@
         <v>18.649999999999999</v>
       </c>
     </row>
-    <row r="96" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
         <v>17</v>
       </c>
@@ -6322,7 +6309,7 @@
         <v>18.55</v>
       </c>
     </row>
-    <row r="97" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>18</v>
       </c>
@@ -6375,7 +6362,7 @@
         <v>18.649999999999999</v>
       </c>
     </row>
-    <row r="98" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>15</v>
       </c>
@@ -6428,7 +6415,7 @@
         <v>19.649999999999999</v>
       </c>
     </row>
-    <row r="99" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
         <v>16</v>
       </c>
@@ -6481,7 +6468,7 @@
         <v>19.600000000000001</v>
       </c>
     </row>
-    <row r="100" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
         <v>17</v>
       </c>
@@ -6534,7 +6521,7 @@
         <v>19.649999999999999</v>
       </c>
     </row>
-    <row r="101" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
         <v>18</v>
       </c>
@@ -6587,7 +6574,7 @@
         <v>19.700000000000003</v>
       </c>
     </row>
-    <row r="102" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>19</v>
       </c>
@@ -6640,7 +6627,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="103" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>20</v>
       </c>
@@ -6693,7 +6680,7 @@
         <v>16.55</v>
       </c>
     </row>
-    <row r="104" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>19</v>
       </c>
@@ -6746,7 +6733,7 @@
         <v>16.75</v>
       </c>
     </row>
-    <row r="105" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>20</v>
       </c>
@@ -6799,7 +6786,7 @@
         <v>16.75</v>
       </c>
     </row>
-    <row r="106" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>19</v>
       </c>
@@ -6852,7 +6839,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="107" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>20</v>
       </c>
@@ -6905,7 +6892,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="108" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>19</v>
       </c>
@@ -6958,7 +6945,7 @@
         <v>19.149999999999999</v>
       </c>
     </row>
-    <row r="109" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>20</v>
       </c>
@@ -7011,7 +6998,7 @@
         <v>19.25</v>
       </c>
     </row>
-    <row r="110" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
         <v>19</v>
       </c>
@@ -7064,7 +7051,7 @@
         <v>18.75</v>
       </c>
     </row>
-    <row r="111" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>20</v>
       </c>
@@ -7117,7 +7104,7 @@
         <v>18.7</v>
       </c>
     </row>
-    <row r="112" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>21</v>
       </c>
@@ -7170,7 +7157,7 @@
         <v>10.7</v>
       </c>
     </row>
-    <row r="113" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>21</v>
       </c>
@@ -7223,7 +7210,7 @@
         <v>11.65</v>
       </c>
     </row>
-    <row r="114" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
         <v>21</v>
       </c>
@@ -7276,7 +7263,7 @@
         <v>13.25</v>
       </c>
     </row>
-    <row r="115" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
         <v>21</v>
       </c>
@@ -7329,7 +7316,7 @@
         <v>16.05</v>
       </c>
     </row>
-    <row r="116" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
         <v>21</v>
       </c>
@@ -7382,7 +7369,7 @@
         <v>18.049999999999997</v>
       </c>
     </row>
-    <row r="117" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
         <v>21</v>
       </c>
@@ -7435,7 +7422,7 @@
         <v>19.350000000000001</v>
       </c>
     </row>
-    <row r="118" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>21</v>
       </c>
@@ -7488,7 +7475,7 @@
         <v>19.45</v>
       </c>
     </row>
-    <row r="119" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B119" t="s">
         <v>22</v>
       </c>
@@ -7541,7 +7528,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="120" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B120" t="s">
         <v>23</v>
       </c>
@@ -7594,7 +7581,7 @@
         <v>15.55</v>
       </c>
     </row>
-    <row r="121" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
         <v>22</v>
       </c>
@@ -7647,7 +7634,7 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="122" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>23</v>
       </c>
@@ -7700,7 +7687,7 @@
         <v>15.950000000000001</v>
       </c>
     </row>
-    <row r="123" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>22</v>
       </c>
@@ -7753,7 +7740,7 @@
         <v>16.600000000000001</v>
       </c>
     </row>
-    <row r="124" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>23</v>
       </c>
@@ -7806,7 +7793,7 @@
         <v>16.649999999999999</v>
       </c>
     </row>
-    <row r="125" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>23</v>
       </c>
@@ -7859,7 +7846,7 @@
         <v>17.549999999999997</v>
       </c>
     </row>
-    <row r="126" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>22</v>
       </c>
@@ -7912,7 +7899,7 @@
         <v>18.850000000000001</v>
       </c>
     </row>
-    <row r="127" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
remove Japan Shapefiles - too big
</commit_message>
<xml_diff>
--- a/Single sheet May2023 Data.xlsx
+++ b/Single sheet May2023 Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heref\Documents\UW Madison Files\Project Stuff\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heref\Documents\Project stuff\LucasProject\Repo_Backup\Project_code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17604571-65B4-4927-988B-9F613E259A2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00CA4BE-EAC7-482E-8543-B5963448F61D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{B2BB9978-D008-4886-AD29-AD3E6970A3E0}"/>
+    <workbookView xWindow="-12105" yWindow="-3900" windowWidth="12210" windowHeight="12885" activeTab="1" xr2:uid="{B2BB9978-D008-4886-AD29-AD3E6970A3E0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -298,14 +298,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -643,177 +642,165 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E27A5A1E-CE4A-441F-B2B9-A3107CDC5860}">
   <dimension ref="A1:G15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5">
         <v>39</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5">
         <v>0.23877614949795342</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5">
         <v>6.1224653717423952E-3</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5">
         <v>5.4937261264824307E-6</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>52</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6">
         <v>71</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6">
         <v>0.54928979571594061</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6">
         <v>7.7364759959991638E-3</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E6">
         <v>2.6705201981185646E-6</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="4">
         <v>16</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <v>6.4935064363996473E-2</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>4.0584415227497795E-3</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <v>1.3250689753439367E-6</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12">
         <v>2.0031291525330795E-4</v>
       </c>
-      <c r="C12" s="4">
+      <c r="C12">
         <v>2</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12">
         <v>1.0015645762665397E-4</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E12">
         <v>29.643921572674078</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F12">
         <v>3.1086040889228957E-11</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12">
         <v>3.0698942378503262</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>63</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13">
         <v>4.155740413047909E-4</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C13">
         <v>123</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D13">
         <v>3.378650742315373E-6</v>
       </c>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-    </row>
-    <row r="15" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="5" t="s">
+    </row>
+    <row r="15" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="4">
         <v>6.1588695655809885E-4</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="4">
         <v>125</v>
       </c>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -824,9 +811,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11F99FF0-2235-4DA3-8ED8-44AD23702AC2}">
   <dimension ref="B1:X127"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -888,7 +875,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>6</v>
       </c>
@@ -950,7 +937,7 @@
         <v>2.1540893888719959E-3</v>
       </c>
     </row>
-    <row r="3" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>7</v>
       </c>
@@ -1015,7 +1002,7 @@
         <v>2.6541458541458523E-3</v>
       </c>
     </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -1081,7 +1068,7 @@
         <v>2.7411670296916164E-3</v>
       </c>
     </row>
-    <row r="5" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>7</v>
       </c>
@@ -1143,7 +1130,7 @@
         <v>4.6043660687138926E-3</v>
       </c>
     </row>
-    <row r="6" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>6</v>
       </c>
@@ -1208,7 +1195,7 @@
         <v>3.7158041958041945E-3</v>
       </c>
     </row>
-    <row r="7" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>7</v>
       </c>
@@ -1274,7 +1261,7 @@
         <v>5.5737062937063148E-3</v>
       </c>
     </row>
-    <row r="8" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>6</v>
       </c>
@@ -1336,7 +1323,7 @@
         <v>4.9262555626191995E-3</v>
       </c>
     </row>
-    <row r="9" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>7</v>
       </c>
@@ -1401,7 +1388,7 @@
         <v>4.2723281250000023E-3</v>
       </c>
     </row>
-    <row r="10" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>6</v>
       </c>
@@ -1467,7 +1454,7 @@
         <v>3.3942770831585146E-3</v>
       </c>
     </row>
-    <row r="11" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>7</v>
       </c>
@@ -1529,7 +1516,7 @@
         <v>4.7151933962264192E-3</v>
       </c>
     </row>
-    <row r="12" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>6</v>
       </c>
@@ -1591,7 +1578,7 @@
         <v>3.2661911554921512E-3</v>
       </c>
     </row>
-    <row r="13" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>7</v>
       </c>
@@ -1653,7 +1640,7 @@
         <v>4.7420048076923021E-3</v>
       </c>
     </row>
-    <row r="14" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>7</v>
       </c>
@@ -1715,7 +1702,7 @@
         <v>4.0199275759903435E-3</v>
       </c>
     </row>
-    <row r="15" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>6</v>
       </c>
@@ -1777,7 +1764,7 @@
         <v>3.6487180475768162E-3</v>
       </c>
     </row>
-    <row r="16" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>6</v>
       </c>
@@ -1839,7 +1826,7 @@
         <v>6.6745588235293928E-3</v>
       </c>
     </row>
-    <row r="17" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>7</v>
       </c>
@@ -1901,7 +1888,7 @@
         <v>3.8323309557774621E-3</v>
       </c>
     </row>
-    <row r="18" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>8</v>
       </c>
@@ -1960,7 +1947,7 @@
         <v>8.3226457590876782E-3</v>
       </c>
     </row>
-    <row r="19" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>9</v>
       </c>
@@ -2019,7 +2006,7 @@
         <v>3.9149065743944575E-3</v>
       </c>
     </row>
-    <row r="20" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>10</v>
       </c>
@@ -2078,7 +2065,7 @@
         <v>9.045566433566422E-3</v>
       </c>
     </row>
-    <row r="21" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>8</v>
       </c>
@@ -2137,7 +2124,7 @@
         <v>6.0018550724637611E-3</v>
       </c>
     </row>
-    <row r="22" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>9</v>
       </c>
@@ -2196,7 +2183,7 @@
         <v>6.2079999999999922E-3</v>
       </c>
     </row>
-    <row r="23" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>10</v>
       </c>
@@ -2255,7 +2242,7 @@
         <v>7.037333333333326E-3</v>
       </c>
     </row>
-    <row r="24" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>8</v>
       </c>
@@ -2314,7 +2301,7 @@
         <v>6.7993043478261021E-3</v>
       </c>
     </row>
-    <row r="25" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>9</v>
       </c>
@@ -2373,7 +2360,7 @@
         <v>6.9125524296675478E-3</v>
       </c>
     </row>
-    <row r="26" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>10</v>
       </c>
@@ -2432,7 +2419,7 @@
         <v>6.1630328820116058E-3</v>
       </c>
     </row>
-    <row r="27" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>8</v>
       </c>
@@ -2491,7 +2478,7 @@
         <v>6.9503999999999989E-3</v>
       </c>
     </row>
-    <row r="28" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>9</v>
       </c>
@@ -2550,7 +2537,7 @@
         <v>1.192713472485772E-2</v>
       </c>
     </row>
-    <row r="29" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
         <v>10</v>
       </c>
@@ -2609,7 +2596,7 @@
         <v>9.258228739002965E-3</v>
       </c>
     </row>
-    <row r="30" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>8</v>
       </c>
@@ -2668,7 +2655,7 @@
         <v>6.8748521739130687E-3</v>
       </c>
     </row>
-    <row r="31" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>9</v>
       </c>
@@ -2727,7 +2714,7 @@
         <v>6.8967619047619272E-3</v>
       </c>
     </row>
-    <row r="32" spans="2:24" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:24" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>10</v>
       </c>
@@ -2786,7 +2773,7 @@
         <v>9.8308571428571429E-3</v>
       </c>
     </row>
-    <row r="33" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>8</v>
       </c>
@@ -2845,7 +2832,7 @@
         <v>6.9470151975684147E-3</v>
       </c>
     </row>
-    <row r="34" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>9</v>
       </c>
@@ -2904,7 +2891,7 @@
         <v>9.9615584415584379E-3</v>
       </c>
     </row>
-    <row r="35" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>10</v>
       </c>
@@ -2963,7 +2950,7 @@
         <v>7.2217600000000033E-3</v>
       </c>
     </row>
-    <row r="36" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>11</v>
       </c>
@@ -3022,7 +3009,7 @@
         <v>8.1333551020408203E-3</v>
       </c>
     </row>
-    <row r="37" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>11</v>
       </c>
@@ -3081,7 +3068,7 @@
         <v>6.8943523404255136E-3</v>
       </c>
     </row>
-    <row r="38" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>11</v>
       </c>
@@ -3140,7 +3127,7 @@
         <v>8.3184872727273037E-3</v>
       </c>
     </row>
-    <row r="39" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>11</v>
       </c>
@@ -3199,7 +3186,7 @@
         <v>6.7314285714285783E-3</v>
       </c>
     </row>
-    <row r="40" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>11</v>
       </c>
@@ -3258,7 +3245,7 @@
         <v>8.1600000000000058E-3</v>
       </c>
     </row>
-    <row r="41" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>12</v>
       </c>
@@ -3314,7 +3301,7 @@
         <v>7.7284578136463675E-3</v>
       </c>
     </row>
-    <row r="42" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>13</v>
       </c>
@@ -3370,7 +3357,7 @@
         <v>1.0947611285266459E-2</v>
       </c>
     </row>
-    <row r="43" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
         <v>14</v>
       </c>
@@ -3426,7 +3413,7 @@
         <v>6.4074830769230758E-3</v>
       </c>
     </row>
-    <row r="44" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B44" t="s">
         <v>14</v>
       </c>
@@ -3482,7 +3469,7 @@
         <v>5.7845106382978725E-3</v>
       </c>
     </row>
-    <row r="45" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B45" t="s">
         <v>12</v>
       </c>
@@ -3538,7 +3525,7 @@
         <v>9.3658181818181765E-3</v>
       </c>
     </row>
-    <row r="46" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B46" t="s">
         <v>13</v>
       </c>
@@ -3594,7 +3581,7 @@
         <v>5.2039344262295112E-3</v>
       </c>
     </row>
-    <row r="47" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B47" t="s">
         <v>12</v>
       </c>
@@ -3650,7 +3637,7 @@
         <v>5.8575238095238159E-3</v>
       </c>
     </row>
-    <row r="48" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B48" t="s">
         <v>14</v>
       </c>
@@ -3706,7 +3693,7 @@
         <v>5.2697806451612889E-3</v>
       </c>
     </row>
-    <row r="49" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B49" t="s">
         <v>14</v>
       </c>
@@ -3762,7 +3749,7 @@
         <v>7.3164255319149015E-3</v>
       </c>
     </row>
-    <row r="50" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B50" t="s">
         <v>12</v>
       </c>
@@ -3818,7 +3805,7 @@
         <v>5.2629482517482524E-3</v>
       </c>
     </row>
-    <row r="51" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B51" t="s">
         <v>13</v>
       </c>
@@ -3874,7 +3861,7 @@
         <v>6.3299047619047579E-3</v>
       </c>
     </row>
-    <row r="52" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B52" t="s">
         <v>12</v>
       </c>
@@ -3930,7 +3917,7 @@
         <v>9.4034285714285661E-3</v>
       </c>
     </row>
-    <row r="53" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B53" t="s">
         <v>14</v>
       </c>
@@ -3986,7 +3973,7 @@
         <v>8.3378797409805749E-3</v>
       </c>
     </row>
-    <row r="54" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B54" t="s">
         <v>13</v>
       </c>
@@ -4042,7 +4029,7 @@
         <v>6.5454545454545453E-3</v>
       </c>
     </row>
-    <row r="55" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B55" t="s">
         <v>12</v>
       </c>
@@ -4098,7 +4085,7 @@
         <v>8.1504864864864815E-3</v>
       </c>
     </row>
-    <row r="56" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B56" t="s">
         <v>13</v>
       </c>
@@ -4154,7 +4141,7 @@
         <v>1.0091935135135129E-2</v>
       </c>
     </row>
-    <row r="57" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B57" t="s">
         <v>14</v>
       </c>
@@ -4210,7 +4197,7 @@
         <v>7.5544367301231723E-3</v>
       </c>
     </row>
-    <row r="58" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B58" t="s">
         <v>12</v>
       </c>
@@ -4266,7 +4253,7 @@
         <v>9.520535885167462E-3</v>
       </c>
     </row>
-    <row r="59" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B59" t="s">
         <v>13</v>
       </c>
@@ -4322,7 +4309,7 @@
         <v>8.6855111111111133E-3</v>
       </c>
     </row>
-    <row r="60" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B60" t="s">
         <v>14</v>
       </c>
@@ -4378,7 +4365,7 @@
         <v>9.778110638297869E-3</v>
       </c>
     </row>
-    <row r="61" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B61" t="s">
         <v>12</v>
       </c>
@@ -4434,7 +4421,7 @@
         <v>8.4756786799826331E-3</v>
       </c>
     </row>
-    <row r="62" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B62" t="s">
         <v>13</v>
       </c>
@@ -4490,7 +4477,7 @@
         <v>8.2873469387754872E-3</v>
       </c>
     </row>
-    <row r="63" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B63" t="s">
         <v>14</v>
       </c>
@@ -4546,7 +4533,7 @@
         <v>6.9284833068362422E-3</v>
       </c>
     </row>
-    <row r="64" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B64" t="s">
         <v>12</v>
       </c>
@@ -4602,7 +4589,7 @@
         <v>6.8520452830188663E-3</v>
       </c>
     </row>
-    <row r="65" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B65" t="s">
         <v>13</v>
       </c>
@@ -4658,7 +4645,7 @@
         <v>7.820940336562986E-3</v>
       </c>
     </row>
-    <row r="66" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B66" t="s">
         <v>14</v>
       </c>
@@ -4714,7 +4701,7 @@
         <v>7.8665890909090964E-3</v>
       </c>
     </row>
-    <row r="67" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B67" t="s">
         <v>12</v>
       </c>
@@ -4770,7 +4757,7 @@
         <v>8.1375135135135206E-3</v>
       </c>
     </row>
-    <row r="68" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B68" t="s">
         <v>13</v>
       </c>
@@ -4826,7 +4813,7 @@
         <v>7.5822545454545514E-3</v>
       </c>
     </row>
-    <row r="69" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B69" t="s">
         <v>14</v>
       </c>
@@ -4882,7 +4869,7 @@
         <v>8.8815021337126671E-3</v>
       </c>
     </row>
-    <row r="70" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B70" t="s">
         <v>15</v>
       </c>
@@ -4938,7 +4925,7 @@
         <v>7.7969230769230763E-3</v>
       </c>
     </row>
-    <row r="71" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B71" t="s">
         <v>16</v>
       </c>
@@ -4994,7 +4981,7 @@
         <v>7.4424092664092684E-3</v>
       </c>
     </row>
-    <row r="72" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B72" t="s">
         <v>17</v>
       </c>
@@ -5050,7 +5037,7 @@
         <v>7.8703058823529209E-3</v>
       </c>
     </row>
-    <row r="73" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B73" t="s">
         <v>18</v>
       </c>
@@ -5103,7 +5090,7 @@
         <v>19.350000000000001</v>
       </c>
     </row>
-    <row r="74" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B74" t="s">
         <v>15</v>
       </c>
@@ -5156,7 +5143,7 @@
         <v>18.55</v>
       </c>
     </row>
-    <row r="75" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B75" t="s">
         <v>16</v>
       </c>
@@ -5209,7 +5196,7 @@
         <v>18.649999999999999</v>
       </c>
     </row>
-    <row r="76" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B76" t="s">
         <v>17</v>
       </c>
@@ -5262,7 +5249,7 @@
         <v>18.799999999999997</v>
       </c>
     </row>
-    <row r="77" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B77" t="s">
         <v>18</v>
       </c>
@@ -5315,7 +5302,7 @@
         <v>18.799999999999997</v>
       </c>
     </row>
-    <row r="78" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B78" t="s">
         <v>15</v>
       </c>
@@ -5368,7 +5355,7 @@
         <v>14.75</v>
       </c>
     </row>
-    <row r="79" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B79" t="s">
         <v>16</v>
       </c>
@@ -5421,7 +5408,7 @@
         <v>14.75</v>
       </c>
     </row>
-    <row r="80" spans="2:23" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:23" x14ac:dyDescent="0.3">
       <c r="B80" t="s">
         <v>17</v>
       </c>
@@ -5474,7 +5461,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="81" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B81" t="s">
         <v>18</v>
       </c>
@@ -5527,7 +5514,7 @@
         <v>14.75</v>
       </c>
     </row>
-    <row r="82" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B82" t="s">
         <v>16</v>
       </c>
@@ -5580,7 +5567,7 @@
         <v>14.6</v>
       </c>
     </row>
-    <row r="83" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
         <v>17</v>
       </c>
@@ -5633,7 +5620,7 @@
         <v>14.55</v>
       </c>
     </row>
-    <row r="84" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
         <v>18</v>
       </c>
@@ -5686,7 +5673,7 @@
         <v>14.65</v>
       </c>
     </row>
-    <row r="85" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>15</v>
       </c>
@@ -5739,7 +5726,7 @@
         <v>14.6</v>
       </c>
     </row>
-    <row r="86" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>15</v>
       </c>
@@ -5792,7 +5779,7 @@
         <v>15.55</v>
       </c>
     </row>
-    <row r="87" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>16</v>
       </c>
@@ -5845,7 +5832,7 @@
         <v>15.600000000000001</v>
       </c>
     </row>
-    <row r="88" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
         <v>17</v>
       </c>
@@ -5898,7 +5885,7 @@
         <v>15.6</v>
       </c>
     </row>
-    <row r="89" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B89" t="s">
         <v>18</v>
       </c>
@@ -5951,7 +5938,7 @@
         <v>15.6</v>
       </c>
     </row>
-    <row r="90" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>15</v>
       </c>
@@ -6004,7 +5991,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="91" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>16</v>
       </c>
@@ -6057,7 +6044,7 @@
         <v>16.950000000000003</v>
       </c>
     </row>
-    <row r="92" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B92" t="s">
         <v>17</v>
       </c>
@@ -6110,7 +6097,7 @@
         <v>17.100000000000001</v>
       </c>
     </row>
-    <row r="93" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>18</v>
       </c>
@@ -6163,7 +6150,7 @@
         <v>17.05</v>
       </c>
     </row>
-    <row r="94" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>15</v>
       </c>
@@ -6216,7 +6203,7 @@
         <v>18.649999999999999</v>
       </c>
     </row>
-    <row r="95" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>16</v>
       </c>
@@ -6269,7 +6256,7 @@
         <v>18.649999999999999</v>
       </c>
     </row>
-    <row r="96" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
         <v>17</v>
       </c>
@@ -6322,7 +6309,7 @@
         <v>18.55</v>
       </c>
     </row>
-    <row r="97" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>18</v>
       </c>
@@ -6375,7 +6362,7 @@
         <v>18.649999999999999</v>
       </c>
     </row>
-    <row r="98" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>15</v>
       </c>
@@ -6428,7 +6415,7 @@
         <v>19.649999999999999</v>
       </c>
     </row>
-    <row r="99" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
         <v>16</v>
       </c>
@@ -6481,7 +6468,7 @@
         <v>19.600000000000001</v>
       </c>
     </row>
-    <row r="100" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
         <v>17</v>
       </c>
@@ -6534,7 +6521,7 @@
         <v>19.649999999999999</v>
       </c>
     </row>
-    <row r="101" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
         <v>18</v>
       </c>
@@ -6587,7 +6574,7 @@
         <v>19.700000000000003</v>
       </c>
     </row>
-    <row r="102" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>19</v>
       </c>
@@ -6640,7 +6627,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="103" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>20</v>
       </c>
@@ -6693,7 +6680,7 @@
         <v>16.55</v>
       </c>
     </row>
-    <row r="104" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>19</v>
       </c>
@@ -6746,7 +6733,7 @@
         <v>16.75</v>
       </c>
     </row>
-    <row r="105" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>20</v>
       </c>
@@ -6799,7 +6786,7 @@
         <v>16.75</v>
       </c>
     </row>
-    <row r="106" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>19</v>
       </c>
@@ -6852,7 +6839,7 @@
         <v>17.3</v>
       </c>
     </row>
-    <row r="107" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>20</v>
       </c>
@@ -6905,7 +6892,7 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="108" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>19</v>
       </c>
@@ -6958,7 +6945,7 @@
         <v>19.149999999999999</v>
       </c>
     </row>
-    <row r="109" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>20</v>
       </c>
@@ -7011,7 +6998,7 @@
         <v>19.25</v>
       </c>
     </row>
-    <row r="110" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
         <v>19</v>
       </c>
@@ -7064,7 +7051,7 @@
         <v>18.75</v>
       </c>
     </row>
-    <row r="111" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>20</v>
       </c>
@@ -7117,7 +7104,7 @@
         <v>18.7</v>
       </c>
     </row>
-    <row r="112" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>21</v>
       </c>
@@ -7170,7 +7157,7 @@
         <v>10.7</v>
       </c>
     </row>
-    <row r="113" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>21</v>
       </c>
@@ -7223,7 +7210,7 @@
         <v>11.65</v>
       </c>
     </row>
-    <row r="114" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
         <v>21</v>
       </c>
@@ -7276,7 +7263,7 @@
         <v>13.25</v>
       </c>
     </row>
-    <row r="115" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
         <v>21</v>
       </c>
@@ -7329,7 +7316,7 @@
         <v>16.05</v>
       </c>
     </row>
-    <row r="116" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
         <v>21</v>
       </c>
@@ -7382,7 +7369,7 @@
         <v>18.049999999999997</v>
       </c>
     </row>
-    <row r="117" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
         <v>21</v>
       </c>
@@ -7435,7 +7422,7 @@
         <v>19.350000000000001</v>
       </c>
     </row>
-    <row r="118" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>21</v>
       </c>
@@ -7488,7 +7475,7 @@
         <v>19.45</v>
       </c>
     </row>
-    <row r="119" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B119" t="s">
         <v>22</v>
       </c>
@@ -7541,7 +7528,7 @@
         <v>14.8</v>
       </c>
     </row>
-    <row r="120" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B120" t="s">
         <v>23</v>
       </c>
@@ -7594,7 +7581,7 @@
         <v>15.55</v>
       </c>
     </row>
-    <row r="121" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
         <v>22</v>
       </c>
@@ -7647,7 +7634,7 @@
         <v>15.5</v>
       </c>
     </row>
-    <row r="122" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>23</v>
       </c>
@@ -7700,7 +7687,7 @@
         <v>15.950000000000001</v>
       </c>
     </row>
-    <row r="123" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>22</v>
       </c>
@@ -7753,7 +7740,7 @@
         <v>16.600000000000001</v>
       </c>
     </row>
-    <row r="124" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>23</v>
       </c>
@@ -7806,7 +7793,7 @@
         <v>16.649999999999999</v>
       </c>
     </row>
-    <row r="125" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>23</v>
       </c>
@@ -7859,7 +7846,7 @@
         <v>17.549999999999997</v>
       </c>
     </row>
-    <row r="126" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>22</v>
       </c>
@@ -7912,7 +7899,7 @@
         <v>18.850000000000001</v>
       </c>
     </row>
-    <row r="127" spans="2:18" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>23</v>
       </c>

</xml_diff>